<commit_message>
feat(Standard): Update in Xbau Standard
</commit_message>
<xml_diff>
--- a/artifacts/xbau/2.6/docs/Mapping 2.6 - Statistiknachrichten (0421-0427).xlsx
+++ b/artifacts/xbau/2.6/docs/Mapping 2.6 - Statistiknachrichten (0421-0427).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://portal.init.de/project/LGV-XBAU/Freigegebene Dokumente/XBau-Dokumente/Arbeitspakete/AP 01 DÜ Statistik/04 Statistikrelevante Daten/Ein- und Ausgangsnachrichten/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\griedel\Documents\XBau\XBau_git\XBau\spezifikation\Ergänzungen\Mappingtabellen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{077109F7-1520-4055-8E22-88106D8C050C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1D548F5-BB48-4ECE-AF07-4B4E6A54AF48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D4DDF000-8FF3-4018-BB4F-E1E0272FCD2A}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D4DDF000-8FF3-4018-BB4F-E1E0272FCD2A}"/>
   </bookViews>
   <sheets>
     <sheet name="0421-0427" sheetId="22" r:id="rId1"/>
@@ -1107,9 +1107,6 @@
     <t>Verwendung in</t>
   </si>
   <si>
-    <t>Der Inhalt der Kindelemente ergibt sich aus dem Datentyp Grundstueck,  GrundstueckStatistik oder DatenBauabgangBeseitungAbsicht der Eingangsnachricht.</t>
-  </si>
-  <si>
     <t>BeteiligteBauprojektStatistik</t>
   </si>
   <si>
@@ -2261,18 +2258,6 @@
       </rPr>
       <t>:statusSozialerWohnungsbau</t>
     </r>
-  </si>
-  <si>
-    <t>0950:datenBauabgang:DatenBauabgangBeseitungAbsicht:bauabgang</t>
-  </si>
-  <si>
-    <t>0950:datenBauabgang:DatenBauabgangBeseitungAbsicht:artDesWohngebaeudes</t>
-  </si>
-  <si>
-    <t>0950:datenBauabgang:DatenBauabgangBeseitungAbsicht:artDesNichtwohngebaeudes</t>
-  </si>
-  <si>
-    <t>0950:datenBauabgang:DatenBauabgangBeseitungAbsicht:ueberbauteFlaeche</t>
   </si>
   <si>
     <t>verortungHausnummer</t>
@@ -3156,13 +3141,6 @@
       </rPr>
       <t>:anzahlDerWohnungen</t>
     </r>
-  </si>
-  <si>
-    <t>Der Inhalt des Elements ergibt sich aus dem Datentyp DatenEinzelnesGebaeudeImBauvorhaben oder DatenBauabgangBeseitungAbsicht der Eingangsnachricht.</t>
-  </si>
-  <si>
-    <t>0420:bauvorhabenGebaeude:datenEinzelnesGebaeude:lageGebaeude
-0950:datenBauabgang:DatenBauabgangBeseitungAbsicht:lageGebaeude</t>
   </si>
   <si>
     <t>0420:bauvorhabenGebaeude:datenEinzelnesGebaeude:artDesBauens</t>
@@ -3827,84 +3805,106 @@
     </r>
   </si>
   <si>
+    <t>0421 - 0427: allgemeineAngaben:baugrundstueck:anschrift</t>
+  </si>
+  <si>
+    <t>0421 - 0427: allgemeineAngaben:baugrundstueck:flurstueck</t>
+  </si>
+  <si>
+    <r>
+      <t>0950:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>anzeigender</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:artDesAnzeigenden</t>
+    </r>
+  </si>
+  <si>
+    <t>0950:anzeigender:AnzeigenderBeseitigung:artDesAnzeigenden</t>
+  </si>
+  <si>
+    <t>Der Inhalt des Elements ergibt sich aus dem Inhalt des Elements "artDesAnzeigenden" im Datentyp AnzeigenderBeseitigung der Eingangsnachricht.</t>
+  </si>
+  <si>
+    <t>0426: datenBauabgang:artDesEigentuemers</t>
+  </si>
+  <si>
+    <t>AmBauBeteiligtePerson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0420:ansprechpartner:datenAnsprechpartner:bevollmaechtigter
+</t>
+  </si>
+  <si>
+    <t>0420:ansprechpartner:datenAnsprechpartner:architektEntwurfsverfasser</t>
+  </si>
+  <si>
+    <t>Der Inhalt des Elements ergibt sich aus dem Datentyp datenAnsprechpartner der Eingangsnachricht.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0420:ansprechpartner:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>datenAnsprechpartner</t>
+    </r>
+  </si>
+  <si>
     <t>0200:bauvorhaben:verortung:baugrundstueck:grundstueck
 0420:allgemeineAngaben:baugrundstueck:GrundstueckStatistik
 0600:bauvorhaben:verortung:baugrundstueck:grundstueck
-0950:datenBauabgang:DatenBauabgangBeseitungAbsicht</t>
-  </si>
-  <si>
-    <t>0421 - 0427: allgemeineAngaben:baugrundstueck:anschrift</t>
-  </si>
-  <si>
-    <t>0421 - 0427: allgemeineAngaben:baugrundstueck:flurstueck</t>
-  </si>
-  <si>
-    <r>
-      <t>0950:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>anzeigender</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>:artDesAnzeigenden</t>
-    </r>
-  </si>
-  <si>
-    <t>0950:anzeigender:AnzeigenderBeseitigung:artDesAnzeigenden</t>
-  </si>
-  <si>
-    <t>Der Inhalt des Elements ergibt sich aus dem Inhalt des Elements "artDesAnzeigenden" im Datentyp AnzeigenderBeseitigung der Eingangsnachricht.</t>
-  </si>
-  <si>
-    <t>0426: datenBauabgang:artDesEigentuemers</t>
-  </si>
-  <si>
-    <t>AmBauBeteiligtePerson</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0420:ansprechpartner:datenAnsprechpartner:bevollmaechtigter
-</t>
-  </si>
-  <si>
-    <t>0420:ansprechpartner:datenAnsprechpartner:architektEntwurfsverfasser</t>
-  </si>
-  <si>
-    <t>Der Inhalt des Elements ergibt sich aus dem Datentyp datenAnsprechpartner der Eingangsnachricht.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0420:ansprechpartner:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>datenAnsprechpartner</t>
-    </r>
+0950:datenBauabgang:DatenBauabgangBeseitigungAbsicht</t>
+  </si>
+  <si>
+    <t>Der Inhalt der Kindelemente ergibt sich aus dem Datentyp Grundstueck,  GrundstueckStatistik oder DatenBauabgangBeseitigungAbsicht der Eingangsnachricht.</t>
+  </si>
+  <si>
+    <t>0420:bauvorhabenGebaeude:datenEinzelnesGebaeude:lageGebaeude
+0950:datenBauabgang:DatenBauabgangBeseitigungAbsicht:lageGebaeude</t>
+  </si>
+  <si>
+    <t>Der Inhalt des Elements ergibt sich aus dem Datentyp DatenEinzelnesGebaeudeImBauvorhaben oder DatenBauabgangBeseitigungAbsicht der Eingangsnachricht.</t>
+  </si>
+  <si>
+    <t>0950:datenBauabgang:DatenBauabgangBeseitigungAbsicht:bauabgang</t>
+  </si>
+  <si>
+    <t>0950:datenBauabgang:DatenBauabgangBeseitigungAbsicht:artDesWohngebaeudes</t>
+  </si>
+  <si>
+    <t>0950:datenBauabgang:DatenBauabgangBeseitigungAbsicht:artDesNichtwohngebaeudes</t>
+  </si>
+  <si>
+    <t>0950:datenBauabgang:DatenBauabgangBeseitigungAbsicht:ueberbauteFlaeche</t>
   </si>
 </sst>
 </file>
@@ -4301,7 +4301,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="168">
+  <cellXfs count="166">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -4742,12 +4742,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -5068,34 +5062,34 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D00349E4-F40C-4C71-9206-95636ED6063A}">
   <dimension ref="A1:F80"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="66.140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="34.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="66.1796875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="34.1796875" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="104" style="2" customWidth="1"/>
-    <col min="4" max="4" width="87.42578125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="21.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="1.28515625" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="11.42578125" style="1"/>
+    <col min="4" max="4" width="87.453125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="21.1796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="1.26953125" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="11.453125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" customFormat="1" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="11" t="s">
-        <v>480</v>
+        <v>475</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="14"/>
       <c r="D1" s="14"/>
       <c r="E1" s="77"/>
     </row>
-    <row r="2" spans="1:5" customFormat="1" ht="21" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A2" s="11"/>
       <c r="B2" s="2"/>
       <c r="C2" s="14"/>
       <c r="D2" s="14"/>
       <c r="E2" s="77"/>
     </row>
-    <row r="3" spans="1:5" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" s="36" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="34" t="s">
         <v>1</v>
       </c>
@@ -5112,7 +5106,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="45" t="s">
         <v>274</v>
       </c>
@@ -5123,7 +5117,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="39" t="s">
         <v>272</v>
       </c>
@@ -5131,14 +5125,14 @@
         <v>273</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>523</v>
+        <v>516</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>276</v>
       </c>
       <c r="E5" s="24"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="45" t="s">
         <v>105</v>
       </c>
@@ -5149,37 +5143,37 @@
         <v>291</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="58" x14ac:dyDescent="0.35">
       <c r="A7" s="17" t="s">
         <v>253</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C7" s="97" t="s">
-        <v>524</v>
+        <v>517</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>277</v>
       </c>
       <c r="E7" s="24"/>
     </row>
-    <row r="8" spans="1:5" ht="90" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="87" x14ac:dyDescent="0.35">
       <c r="A8" s="83" t="s">
-        <v>475</v>
+        <v>470</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C8" s="97" t="s">
-        <v>502</v>
+        <v>495</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>433</v>
+        <v>428</v>
       </c>
       <c r="E8" s="24"/>
     </row>
-    <row r="9" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="58" x14ac:dyDescent="0.35">
       <c r="A9" s="17" t="s">
         <v>119</v>
       </c>
@@ -5187,14 +5181,14 @@
         <v>245</v>
       </c>
       <c r="C9" s="97" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>308</v>
+        <v>543</v>
       </c>
       <c r="E9" s="24"/>
     </row>
-    <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="17" t="s">
         <v>254</v>
       </c>
@@ -5202,14 +5196,14 @@
         <v>20</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>489</v>
+        <v>544</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>488</v>
+        <v>545</v>
       </c>
       <c r="E10" s="24"/>
     </row>
-    <row r="11" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="18" t="s">
         <v>120</v>
       </c>
@@ -5224,7 +5218,7 @@
       </c>
       <c r="E11" s="50"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="41" t="s">
         <v>8</v>
       </c>
@@ -5234,7 +5228,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="17" t="s">
         <v>124</v>
       </c>
@@ -5249,7 +5243,7 @@
       </c>
       <c r="E13" s="42"/>
     </row>
-    <row r="14" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="17" t="s">
         <v>255</v>
       </c>
@@ -5264,7 +5258,7 @@
       </c>
       <c r="E14" s="24"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="45" t="s">
         <v>182</v>
       </c>
@@ -5275,7 +5269,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="17" t="s">
         <v>174</v>
       </c>
@@ -5290,7 +5284,7 @@
       </c>
       <c r="E16" s="24"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="17" t="s">
         <v>175</v>
       </c>
@@ -5305,7 +5299,7 @@
       </c>
       <c r="E17" s="24"/>
     </row>
-    <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="17" t="s">
         <v>176</v>
       </c>
@@ -5313,14 +5307,14 @@
         <v>42</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>372</v>
+        <v>546</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="E18" s="24"/>
     </row>
-    <row r="19" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="17" t="s">
         <v>177</v>
       </c>
@@ -5328,14 +5322,14 @@
         <v>43</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>542</v>
+        <v>534</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>543</v>
+        <v>535</v>
       </c>
       <c r="E19" s="24"/>
     </row>
-    <row r="20" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="17" t="s">
         <v>248</v>
       </c>
@@ -5343,14 +5337,14 @@
         <v>28</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>373</v>
+        <v>547</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="E20" s="24"/>
     </row>
-    <row r="21" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="17" t="s">
         <v>179</v>
       </c>
@@ -5358,14 +5352,14 @@
         <v>45</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>374</v>
+        <v>548</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="E21" s="24"/>
     </row>
-    <row r="22" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="17" t="s">
         <v>180</v>
       </c>
@@ -5373,14 +5367,14 @@
         <v>15</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>375</v>
+        <v>549</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="E22" s="24"/>
     </row>
-    <row r="23" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="18" t="s">
         <v>181</v>
       </c>
@@ -5395,7 +5389,7 @@
       </c>
       <c r="E23" s="50"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="41" t="s">
         <v>9</v>
       </c>
@@ -5403,7 +5397,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="17" t="s">
         <v>187</v>
       </c>
@@ -5418,7 +5412,7 @@
       </c>
       <c r="E25" s="24"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="17" t="s">
         <v>185</v>
       </c>
@@ -5433,7 +5427,7 @@
       </c>
       <c r="E26" s="24"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="17" t="s">
         <v>256</v>
       </c>
@@ -5448,7 +5442,7 @@
       </c>
       <c r="E27" s="24"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="17" t="s">
         <v>184</v>
       </c>
@@ -5463,7 +5457,7 @@
       </c>
       <c r="E28" s="24"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="17" t="s">
         <v>240</v>
       </c>
@@ -5478,7 +5472,7 @@
       </c>
       <c r="E29" s="24"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="17" t="s">
         <v>239</v>
       </c>
@@ -5493,7 +5487,7 @@
       </c>
       <c r="E30" s="24"/>
     </row>
-    <row r="31" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="18" t="s">
         <v>257</v>
       </c>
@@ -5508,7 +5502,7 @@
       </c>
       <c r="E31" s="50"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="41" t="s">
         <v>251</v>
       </c>
@@ -5517,7 +5511,7 @@
       </c>
       <c r="F32" s="2"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="17" t="s">
         <v>192</v>
       </c>
@@ -5533,7 +5527,7 @@
       <c r="E33" s="24"/>
       <c r="F33" s="2"/>
     </row>
-    <row r="34" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="17" t="s">
         <v>258</v>
       </c>
@@ -5548,7 +5542,7 @@
       </c>
       <c r="E34" s="24"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="21" t="s">
         <v>14</v>
       </c>
@@ -5565,7 +5559,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" s="56" t="s">
         <v>12</v>
       </c>
@@ -5580,7 +5574,7 @@
       </c>
       <c r="E36" s="78"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" s="41" t="s">
         <v>259</v>
       </c>
@@ -5589,7 +5583,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" s="47" t="s">
         <v>241</v>
       </c>
@@ -5604,7 +5598,7 @@
       </c>
       <c r="E38" s="24"/>
     </row>
-    <row r="39" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="47" t="s">
         <v>242</v>
       </c>
@@ -5619,7 +5613,7 @@
       </c>
       <c r="E39" s="24"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" s="40" t="s">
         <v>260</v>
       </c>
@@ -5630,7 +5624,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" s="17" t="s">
         <v>261</v>
       </c>
@@ -5645,7 +5639,7 @@
       </c>
       <c r="E41" s="24"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" s="17" t="s">
         <v>262</v>
       </c>
@@ -5660,7 +5654,7 @@
       </c>
       <c r="E42" s="24"/>
     </row>
-    <row r="43" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A43" s="17" t="s">
         <v>292</v>
       </c>
@@ -5668,31 +5662,31 @@
         <v>293</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>490</v>
+        <v>483</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>491</v>
+        <v>484</v>
       </c>
       <c r="E43" s="24"/>
     </row>
-    <row r="44" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" ht="29" x14ac:dyDescent="0.35">
       <c r="A44" s="83" t="s">
-        <v>476</v>
+        <v>471</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>301</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>499</v>
+        <v>492</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>303</v>
       </c>
       <c r="E44" s="24"/>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" s="83" t="s">
-        <v>477</v>
+        <v>472</v>
       </c>
       <c r="B45" s="13" t="s">
         <v>5</v>
@@ -5705,22 +5699,22 @@
       </c>
       <c r="E45" s="24"/>
     </row>
-    <row r="46" spans="1:6" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" ht="78.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="83" t="s">
+        <v>309</v>
+      </c>
+      <c r="B46" s="13" t="s">
         <v>310</v>
       </c>
-      <c r="B46" s="13" t="s">
-        <v>311</v>
-      </c>
       <c r="C46" s="13" t="s">
-        <v>525</v>
+        <v>518</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>492</v>
+        <v>485</v>
       </c>
       <c r="E46" s="24"/>
     </row>
-    <row r="47" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A47" s="83" t="s">
         <v>263</v>
       </c>
@@ -5728,29 +5722,29 @@
         <v>31</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>526</v>
+        <v>519</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="E47" s="24"/>
     </row>
-    <row r="48" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A48" s="83" t="s">
-        <v>478</v>
+        <v>473</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>305</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>527</v>
+        <v>520</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>493</v>
+        <v>486</v>
       </c>
       <c r="E48" s="24"/>
     </row>
-    <row r="49" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A49" s="83" t="s">
         <v>264</v>
       </c>
@@ -5758,14 +5752,14 @@
         <v>34</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>528</v>
+        <v>521</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
       <c r="E49" s="24"/>
     </row>
-    <row r="50" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A50" s="83" t="s">
         <v>265</v>
       </c>
@@ -5773,14 +5767,14 @@
         <v>35</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>529</v>
+        <v>522</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
       <c r="E50" s="24"/>
     </row>
-    <row r="51" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A51" s="83" t="s">
         <v>286</v>
       </c>
@@ -5788,14 +5782,14 @@
         <v>284</v>
       </c>
       <c r="C51" s="13" t="s">
-        <v>494</v>
+        <v>487</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>495</v>
+        <v>488</v>
       </c>
       <c r="E51" s="24"/>
     </row>
-    <row r="52" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A52" s="83" t="s">
         <v>266</v>
       </c>
@@ -5803,14 +5797,14 @@
         <v>17</v>
       </c>
       <c r="C52" s="13" t="s">
-        <v>530</v>
+        <v>523</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>431</v>
+        <v>426</v>
       </c>
       <c r="E52" s="24"/>
     </row>
-    <row r="53" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A53" s="83" t="s">
         <v>267</v>
       </c>
@@ -5818,44 +5812,44 @@
         <v>36</v>
       </c>
       <c r="C53" s="13" t="s">
-        <v>531</v>
+        <v>524</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>304</v>
       </c>
       <c r="E53" s="24"/>
     </row>
-    <row r="54" spans="1:5" ht="105" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A54" s="83" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C54" s="13" t="s">
-        <v>532</v>
+        <v>525</v>
       </c>
       <c r="D54" s="13" t="s">
-        <v>496</v>
+        <v>489</v>
       </c>
       <c r="E54" s="24"/>
     </row>
-    <row r="55" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A55" s="83" t="s">
-        <v>479</v>
+        <v>474</v>
       </c>
       <c r="B55" s="13" t="s">
         <v>302</v>
       </c>
       <c r="C55" s="13" t="s">
-        <v>533</v>
+        <v>526</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>486</v>
+        <v>481</v>
       </c>
       <c r="E55" s="24"/>
     </row>
-    <row r="56" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A56" s="83" t="s">
         <v>287</v>
       </c>
@@ -5863,14 +5857,14 @@
         <v>289</v>
       </c>
       <c r="C56" s="13" t="s">
-        <v>534</v>
+        <v>527</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>290</v>
       </c>
       <c r="E56" s="24"/>
     </row>
-    <row r="57" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A57" s="83" t="s">
         <v>288</v>
       </c>
@@ -5878,14 +5872,14 @@
         <v>282</v>
       </c>
       <c r="C57" s="13" t="s">
-        <v>535</v>
+        <v>528</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>432</v>
+        <v>427</v>
       </c>
       <c r="E57" s="24"/>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="17" t="s">
         <v>268</v>
       </c>
@@ -5900,7 +5894,7 @@
       </c>
       <c r="E58" s="24"/>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="17" t="s">
         <v>269</v>
       </c>
@@ -5915,7 +5909,7 @@
       </c>
       <c r="E59" s="24"/>
     </row>
-    <row r="60" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A60" s="17" t="s">
         <v>270</v>
       </c>
@@ -5923,14 +5917,14 @@
         <v>271</v>
       </c>
       <c r="C60" s="13" t="s">
-        <v>497</v>
+        <v>490</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>498</v>
+        <v>491</v>
       </c>
       <c r="E60" s="24"/>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="53" t="s">
         <v>171</v>
       </c>
@@ -5943,7 +5937,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="39" t="s">
         <v>252</v>
       </c>
@@ -5958,37 +5952,37 @@
       </c>
       <c r="E62" s="24"/>
     </row>
-    <row r="63" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A63" s="39" t="s">
         <v>243</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>545</v>
+        <v>537</v>
       </c>
       <c r="C63" s="13" t="s">
-        <v>546</v>
-      </c>
-      <c r="D63" s="166" t="s">
-        <v>548</v>
+        <v>538</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>540</v>
       </c>
       <c r="E63" s="24"/>
     </row>
-    <row r="64" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A64" s="22" t="s">
         <v>244</v>
       </c>
       <c r="B64" s="20" t="s">
-        <v>545</v>
+        <v>537</v>
       </c>
       <c r="C64" s="31" t="s">
-        <v>547</v>
-      </c>
-      <c r="D64" s="167" t="s">
-        <v>548</v>
+        <v>539</v>
+      </c>
+      <c r="D64" s="20" t="s">
+        <v>540</v>
       </c>
       <c r="E64" s="50"/>
     </row>
-    <row r="80" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A80" s="1"/>
       <c r="C80" s="4"/>
       <c r="D80" s="4"/>
@@ -6004,146 +5998,146 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAAE0A6E-F4FA-46B5-980B-7D8FE5FA0DFB}">
   <dimension ref="A1:I29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="127.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="40.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="94.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="127.54296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.453125" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="94.26953125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.54296875" style="4" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="24" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="2.85546875" style="4" customWidth="1"/>
-    <col min="7" max="7" width="31.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="31.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="39.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="10" max="19" width="11.42578125" style="2"/>
-    <col min="20" max="20" width="11.42578125" style="2" customWidth="1"/>
-    <col min="21" max="16384" width="11.42578125" style="2"/>
+    <col min="6" max="6" width="2.81640625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="31.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="31.54296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="39.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="19" width="11.453125" style="2"/>
+    <col min="20" max="20" width="11.453125" style="2" customWidth="1"/>
+    <col min="21" max="16384" width="11.453125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
-        <v>440</v>
+        <v>435</v>
       </c>
       <c r="B1" s="12"/>
     </row>
-    <row r="2" spans="1:3" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="19" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="48" t="s">
-        <v>485</v>
+        <v>480</v>
       </c>
       <c r="B2" s="48"/>
       <c r="C2" s="15"/>
     </row>
-    <row r="3" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="51" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="119" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C3" s="52" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="123" t="s">
-        <v>439</v>
+        <v>434</v>
       </c>
       <c r="B4" s="124" t="s">
         <v>23</v>
       </c>
       <c r="C4" s="125" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="129" t="s">
-        <v>436</v>
+        <v>431</v>
       </c>
       <c r="B5" s="120" t="s">
         <v>24</v>
       </c>
       <c r="C5" s="126" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="122" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="B6" s="136" t="s">
         <v>24</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="138" t="s">
-        <v>438</v>
+        <v>433</v>
       </c>
       <c r="B7" s="137" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="C7" s="139" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="122" t="s">
-        <v>435</v>
+        <v>430</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>273</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="122" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="16" t="s">
-        <v>420</v>
+        <v>415</v>
       </c>
       <c r="B10" s="111" t="s">
         <v>28</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="22" t="s">
-        <v>421</v>
+        <v>416</v>
       </c>
       <c r="B11" s="115" t="s">
         <v>29</v>
       </c>
       <c r="C11" s="38" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="83" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
       <c r="C12" s="121" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="47" t="s">
         <v>236</v>
       </c>
@@ -6151,54 +6145,54 @@
         <v>39</v>
       </c>
       <c r="C13" s="30" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="83" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
       <c r="B14" s="13" t="s">
         <v>289</v>
       </c>
       <c r="C14" s="30" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="47" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="B15" s="140" t="s">
         <v>285</v>
       </c>
       <c r="C15" s="30" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="83" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="B16" s="13" t="s">
         <v>17</v>
       </c>
       <c r="C16" s="30" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="47" t="s">
         <v>237</v>
       </c>
       <c r="B17" s="140" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
       <c r="C17" s="30" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="116" t="s">
         <v>232</v>
       </c>
@@ -6206,21 +6200,21 @@
         <v>31</v>
       </c>
       <c r="C18" s="127" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="39" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>39</v>
       </c>
       <c r="C19" s="30" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" s="17" t="s">
         <v>234</v>
       </c>
@@ -6228,10 +6222,10 @@
         <v>32</v>
       </c>
       <c r="C20" s="30" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="17" t="s">
         <v>235</v>
       </c>
@@ -6239,10 +6233,10 @@
         <v>34</v>
       </c>
       <c r="C21" s="30" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="39" t="s">
         <v>233</v>
       </c>
@@ -6250,76 +6244,76 @@
         <v>35</v>
       </c>
       <c r="C22" s="30" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" s="39" t="s">
-        <v>487</v>
+        <v>482</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>281</v>
       </c>
       <c r="C23" s="30" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" s="128" t="s">
-        <v>398</v>
+        <v>393</v>
       </c>
       <c r="B24" s="94" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C24" s="126" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" s="17" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>39</v>
       </c>
       <c r="C25" s="24" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" s="17" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>39</v>
       </c>
       <c r="C26" s="24" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" s="129" t="s">
-        <v>402</v>
+        <v>397</v>
       </c>
       <c r="B27" s="120" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C27" s="126" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="130" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="B28" s="131" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C28" s="50" t="s">
-        <v>540</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
     </row>
@@ -6332,276 +6326,276 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{160416BC-7406-4B11-BD0B-A0CFC0026B6B}">
   <dimension ref="A1:E24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="87.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="56.5703125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="90.7109375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="79.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="65.7109375" style="2" customWidth="1"/>
-    <col min="6" max="6" width="1.28515625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="14.140625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="67.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="11.42578125" style="1"/>
+    <col min="1" max="1" width="87.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="56.54296875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="90.7265625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="79.1796875" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="65.7265625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="1.26953125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="14.1796875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="67.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="11.453125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" customFormat="1" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="11" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="4"/>
       <c r="E1" s="14"/>
     </row>
-    <row r="2" spans="1:5" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" customFormat="1" ht="18.5" x14ac:dyDescent="0.35">
       <c r="A2" s="49" t="s">
-        <v>484</v>
+        <v>479</v>
       </c>
       <c r="B2" s="49"/>
       <c r="C2" s="88"/>
     </row>
-    <row r="3" spans="1:5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="84" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C3" s="89" t="s">
         <v>110</v>
       </c>
       <c r="D3" s="5"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="85" t="s">
+        <v>351</v>
+      </c>
+      <c r="B4" s="94" t="s">
+        <v>330</v>
+      </c>
+      <c r="C4" s="141" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="8" t="s">
         <v>352</v>
       </c>
-      <c r="B4" s="94" t="s">
-        <v>331</v>
-      </c>
-      <c r="C4" s="141" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+      <c r="B5" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="C5" s="142" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="9" t="s">
         <v>353</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="C5" s="142" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
-        <v>354</v>
       </c>
       <c r="B6" s="95" t="s">
         <v>245</v>
       </c>
       <c r="C6" s="143" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" customFormat="1" x14ac:dyDescent="0.25">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C7" s="142" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="8" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>273</v>
       </c>
       <c r="C8" s="144" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>293</v>
       </c>
       <c r="C9" s="145" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>27</v>
       </c>
       <c r="C10" s="145" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
+        <v>358</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="C11" s="145" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" s="8" t="s">
         <v>359</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>347</v>
-      </c>
-      <c r="C11" s="145" t="s">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
-        <v>360</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>31</v>
       </c>
       <c r="C12" s="145" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="8" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>305</v>
       </c>
       <c r="C13" s="146" t="s">
-        <v>443</v>
+        <v>438</v>
       </c>
       <c r="D13" s="4"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="8" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C14" s="145" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="8" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C15" s="145" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="8" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>284</v>
       </c>
       <c r="C16" s="145" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="8" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>17</v>
       </c>
       <c r="C17" s="145" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="8" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>39</v>
       </c>
       <c r="C18" s="145" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="8" t="s">
+        <v>366</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="C19" s="145" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" s="8" t="s">
         <v>367</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>348</v>
-      </c>
-      <c r="C19" s="145" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="s">
-        <v>368</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>302</v>
       </c>
       <c r="C20" s="145" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="8" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>289</v>
       </c>
       <c r="C21" s="145" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="8" t="s">
+        <v>369</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="C22" s="145" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" s="9" t="s">
         <v>370</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>349</v>
-      </c>
-      <c r="C22" s="145" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="9" t="s">
-        <v>371</v>
       </c>
       <c r="B23" s="95" t="s">
         <v>271</v>
       </c>
       <c r="C23" s="147" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" s="96" t="s">
-        <v>549</v>
+        <v>541</v>
       </c>
       <c r="B24" s="95" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C24" s="143" t="s">
-        <v>446</v>
+        <v>441</v>
       </c>
     </row>
   </sheetData>
@@ -6613,267 +6607,267 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9223024-ADE7-4E5A-950B-375CE0F82733}">
   <dimension ref="A1:I25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="102.85546875" customWidth="1"/>
-    <col min="2" max="2" width="33.42578125" customWidth="1"/>
-    <col min="3" max="3" width="107.85546875" style="66" customWidth="1"/>
-    <col min="4" max="6" width="41.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="102.81640625" customWidth="1"/>
+    <col min="2" max="2" width="33.453125" customWidth="1"/>
+    <col min="3" max="3" width="107.81640625" style="66" customWidth="1"/>
+    <col min="4" max="6" width="41.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="11" t="s">
-        <v>500</v>
+        <v>493</v>
       </c>
       <c r="B1" s="11"/>
     </row>
-    <row r="2" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="18.5" x14ac:dyDescent="0.35">
       <c r="A2" s="49" t="s">
-        <v>501</v>
+        <v>494</v>
       </c>
       <c r="B2" s="49"/>
       <c r="C2" s="88"/>
     </row>
-    <row r="3" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="7" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="84" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C3" s="89" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="158" t="s">
-        <v>503</v>
+        <v>496</v>
       </c>
       <c r="B4" s="159" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C4" s="160" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="162" t="s">
-        <v>504</v>
+        <v>497</v>
       </c>
       <c r="B5" s="44" t="s">
         <v>273</v>
       </c>
       <c r="C5" s="157" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="122" t="s">
-        <v>505</v>
+        <v>498</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="116" t="s">
-        <v>506</v>
+        <v>499</v>
       </c>
       <c r="B7" s="86" t="s">
         <v>28</v>
       </c>
       <c r="C7" s="127" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="114" t="s">
-        <v>507</v>
+        <v>500</v>
       </c>
       <c r="B8" s="87" t="s">
         <v>29</v>
       </c>
       <c r="C8" s="161" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="83" t="s">
-        <v>508</v>
+        <v>501</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
       <c r="C9" s="121" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="47" t="s">
-        <v>509</v>
+        <v>502</v>
       </c>
       <c r="B10" s="140" t="s">
         <v>39</v>
       </c>
       <c r="C10" s="30" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="83" t="s">
-        <v>510</v>
+        <v>503</v>
       </c>
       <c r="B11" s="13" t="s">
         <v>289</v>
       </c>
       <c r="C11" s="30" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="47" t="s">
-        <v>511</v>
+        <v>504</v>
       </c>
       <c r="B12" s="140" t="s">
         <v>285</v>
       </c>
       <c r="C12" s="30" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="83" t="s">
-        <v>512</v>
+        <v>505</v>
       </c>
       <c r="B13" s="13" t="s">
         <v>17</v>
       </c>
       <c r="C13" s="30" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="47" t="s">
-        <v>513</v>
+        <v>506</v>
       </c>
       <c r="B14" s="140" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
       <c r="C14" s="30" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="116" t="s">
-        <v>514</v>
+        <v>507</v>
       </c>
       <c r="B15" s="86" t="s">
         <v>31</v>
       </c>
       <c r="C15" s="127" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="39" t="s">
-        <v>515</v>
+        <v>508</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>39</v>
       </c>
       <c r="C16" s="30" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="17" t="s">
-        <v>516</v>
+        <v>509</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C17" s="30" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="17" t="s">
-        <v>517</v>
+        <v>510</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C18" s="30" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" s="39" t="s">
-        <v>518</v>
+        <v>511</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>35</v>
       </c>
       <c r="C19" s="30" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" s="114" t="s">
-        <v>519</v>
+        <v>512</v>
       </c>
       <c r="B20" s="87" t="s">
         <v>281</v>
       </c>
       <c r="C20" s="161" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="17" t="s">
-        <v>520</v>
+        <v>513</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C21" s="24" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="17" t="s">
-        <v>521</v>
+        <v>514</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>39</v>
       </c>
       <c r="C22" s="24" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="18" t="s">
-        <v>522</v>
+        <v>515</v>
       </c>
       <c r="B23" s="20" t="s">
         <v>39</v>
       </c>
       <c r="C23" s="50" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A24" s="129" t="s">
-        <v>536</v>
+        <v>529</v>
       </c>
       <c r="B24" s="120" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C24" s="126" t="s">
-        <v>539</v>
+        <v>531</v>
       </c>
       <c r="D24" s="4"/>
       <c r="E24" s="4"/>
@@ -6882,15 +6876,15 @@
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
     </row>
-    <row r="25" spans="1:9" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" s="2" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A25" s="130" t="s">
-        <v>537</v>
+        <v>530</v>
       </c>
       <c r="B25" s="131" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C25" s="50" t="s">
-        <v>540</v>
+        <v>532</v>
       </c>
       <c r="D25" s="4"/>
       <c r="E25" s="4"/>
@@ -6908,61 +6902,61 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33E2EA96-3E9F-4F28-AFF4-C694581B8DCB}">
   <dimension ref="A1:E39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="102.85546875" customWidth="1"/>
-    <col min="2" max="2" width="33.42578125" customWidth="1"/>
-    <col min="3" max="3" width="107.85546875" style="66" customWidth="1"/>
-    <col min="4" max="6" width="41.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="102.81640625" customWidth="1"/>
+    <col min="2" max="2" width="33.453125" customWidth="1"/>
+    <col min="3" max="3" width="107.81640625" style="66" customWidth="1"/>
+    <col min="4" max="6" width="41.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="11" t="s">
         <v>247</v>
       </c>
       <c r="B1" s="11"/>
     </row>
-    <row r="2" spans="1:5" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="18.5" x14ac:dyDescent="0.35">
       <c r="A2" s="49" t="s">
-        <v>481</v>
+        <v>476</v>
       </c>
       <c r="B2" s="49"/>
       <c r="C2" s="88"/>
     </row>
-    <row r="3" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="7" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="84" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C3" s="89" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="16" t="s">
-        <v>473</v>
+        <v>468</v>
       </c>
       <c r="B4" s="111" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="152" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="112" t="s">
-        <v>474</v>
+        <v>469</v>
       </c>
       <c r="B5" s="113" t="s">
         <v>271</v>
       </c>
       <c r="C5" s="155" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="21" x14ac:dyDescent="0.35">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="21" x14ac:dyDescent="0.5">
       <c r="A7" s="11" t="s">
         <v>54</v>
       </c>
@@ -6970,325 +6964,325 @@
       <c r="C7" s="4"/>
       <c r="E7" s="14"/>
     </row>
-    <row r="8" spans="1:5" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="18.5" x14ac:dyDescent="0.35">
       <c r="A8" s="49" t="s">
-        <v>482</v>
+        <v>477</v>
       </c>
       <c r="B8" s="49"/>
       <c r="C8" s="88"/>
     </row>
-    <row r="9" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="7" t="s">
         <v>1</v>
       </c>
       <c r="B9" s="84" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C9" s="89" t="s">
         <v>110</v>
       </c>
       <c r="D9" s="5"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="16" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B10" s="111" t="s">
         <v>48</v>
       </c>
       <c r="C10" s="152" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="39" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C11" s="153" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="39" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C12" s="153" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="39" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C13" s="153" t="s">
-        <v>460</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="39" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C14" s="153" t="s">
-        <v>461</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="39" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C15" s="153" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="39" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C16" s="153" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="39" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C17" s="153" t="s">
-        <v>464</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="39" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C18" s="153" t="s">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="39" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C19" s="153" t="s">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" s="39" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C20" s="153" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="39" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C21" s="153" t="s">
-        <v>468</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="114" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B22" s="87" t="s">
         <v>48</v>
       </c>
       <c r="C22" s="154" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="22" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B23" s="115" t="s">
         <v>48</v>
       </c>
       <c r="C23" s="155" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="21" x14ac:dyDescent="0.35">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="21" x14ac:dyDescent="0.5">
       <c r="A25" s="11" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B25" s="11"/>
     </row>
-    <row r="26" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" ht="18.5" x14ac:dyDescent="0.35">
       <c r="A26" s="49" t="s">
-        <v>483</v>
+        <v>478</v>
       </c>
       <c r="B26" s="49"/>
       <c r="C26" s="88"/>
     </row>
-    <row r="27" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="91" t="s">
         <v>1</v>
       </c>
       <c r="B27" s="91" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C27" s="92" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" s="163" t="s">
-        <v>541</v>
+        <v>533</v>
       </c>
       <c r="B28" s="164" t="s">
         <v>43</v>
       </c>
       <c r="C28" s="165" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" s="114" t="s">
-        <v>472</v>
+        <v>467</v>
       </c>
       <c r="B29" s="95" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C29" s="149" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" s="116" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B30" s="86" t="s">
         <v>273</v>
       </c>
       <c r="C30" s="148" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" s="117" t="s">
+        <v>335</v>
+      </c>
+      <c r="B31" s="90" t="s">
+        <v>330</v>
+      </c>
+      <c r="C31" s="149" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32" s="118" t="s">
         <v>336</v>
       </c>
-      <c r="B31" s="90" t="s">
+      <c r="B32" t="s">
+        <v>332</v>
+      </c>
+      <c r="C32" s="150" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" s="118" t="s">
+        <v>337</v>
+      </c>
+      <c r="B33" t="s">
         <v>331</v>
       </c>
-      <c r="C31" s="149" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="118" t="s">
-        <v>337</v>
-      </c>
-      <c r="B32" t="s">
-        <v>333</v>
-      </c>
-      <c r="C32" s="150" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="118" t="s">
+      <c r="C33" s="150" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" s="118" t="s">
         <v>338</v>
-      </c>
-      <c r="B33" t="s">
-        <v>332</v>
-      </c>
-      <c r="C33" s="150" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="118" t="s">
-        <v>339</v>
       </c>
       <c r="B34" t="s">
         <v>20</v>
       </c>
       <c r="C34" s="150" t="s">
-        <v>452</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" s="118" t="s">
+        <v>339</v>
+      </c>
+      <c r="B35" t="s">
+        <v>333</v>
+      </c>
+      <c r="C35" s="150" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36" s="39" t="s">
         <v>340</v>
-      </c>
-      <c r="B35" t="s">
-        <v>334</v>
-      </c>
-      <c r="C35" s="150" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="39" t="s">
-        <v>341</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C36" s="150" t="s">
-        <v>454</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" s="39" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>45</v>
       </c>
       <c r="C37" s="150" t="s">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A38" s="22" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B38" s="20" t="s">
         <v>15</v>
       </c>
       <c r="C38" s="151" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C39" s="2"/>
     </row>
   </sheetData>
@@ -7300,16 +7294,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7397439-CFA1-407D-8F70-92B6FB036848}">
   <dimension ref="A1:G17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="34.7109375" style="66" customWidth="1"/>
-    <col min="2" max="2" width="31.7109375" style="66" customWidth="1"/>
-    <col min="3" max="3" width="24.42578125" style="66" customWidth="1"/>
-    <col min="4" max="4" width="54.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="34.7265625" style="66" customWidth="1"/>
+    <col min="2" max="2" width="31.7265625" style="66" customWidth="1"/>
+    <col min="3" max="3" width="24.453125" style="66" customWidth="1"/>
+    <col min="4" max="4" width="54.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="2" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="2" customFormat="1" ht="18.5" x14ac:dyDescent="0.35">
       <c r="A1" s="48" t="s">
         <v>238</v>
       </c>
@@ -7320,12 +7314,12 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
     </row>
-    <row r="3" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="100" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="101" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C3" s="102" t="s">
         <v>110</v>
@@ -7337,31 +7331,31 @@
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
     </row>
-    <row r="4" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="104" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>48</v>
       </c>
       <c r="C4" s="97" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="D4" s="93"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="104" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>48</v>
       </c>
       <c r="C5" s="97" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="D5" s="93"/>
     </row>
-    <row r="6" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="104" t="s">
         <v>250</v>
       </c>
@@ -7369,14 +7363,14 @@
         <v>48</v>
       </c>
       <c r="C6" s="97" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="D6" s="93"/>
       <c r="E6" s="98"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>280</v>
@@ -7386,9 +7380,9 @@
       </c>
       <c r="D7" s="93"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="8" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>11</v>
@@ -7398,7 +7392,7 @@
       </c>
       <c r="D8" s="93"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="104" t="s">
         <v>12</v>
       </c>
@@ -7410,7 +7404,7 @@
       </c>
       <c r="D9" s="93"/>
     </row>
-    <row r="10" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="104" t="s">
         <v>13</v>
       </c>
@@ -7418,13 +7412,13 @@
         <v>5</v>
       </c>
       <c r="C10" s="97" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="D10" s="93" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="104" t="s">
         <v>212</v>
       </c>
@@ -7432,13 +7426,13 @@
         <v>5</v>
       </c>
       <c r="C11" s="97" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="D11" s="93" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="104" t="s">
         <v>210</v>
       </c>
@@ -7450,7 +7444,7 @@
       </c>
       <c r="D12" s="93"/>
     </row>
-    <row r="13" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A13" s="105" t="s">
         <v>14</v>
       </c>
@@ -7458,11 +7452,11 @@
         <v>7</v>
       </c>
       <c r="C13" s="97" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="D13" s="93"/>
     </row>
-    <row r="14" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="104" t="s">
         <v>211</v>
       </c>
@@ -7470,14 +7464,14 @@
         <v>5</v>
       </c>
       <c r="C14" s="97" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="D14" s="93" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="E14" s="98"/>
     </row>
-    <row r="15" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A15" s="104" t="s">
         <v>10</v>
       </c>
@@ -7485,12 +7479,12 @@
         <v>4</v>
       </c>
       <c r="C15" s="107" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="D15" s="93"/>
       <c r="E15" s="98"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="108" t="s">
         <v>249</v>
       </c>
@@ -7498,14 +7492,14 @@
         <v>25</v>
       </c>
       <c r="C16" s="107" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="D16" s="93"/>
       <c r="E16" s="99"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="109" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="B17" s="110" t="s">
         <v>300</v>
@@ -7523,19 +7517,19 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F212F51-3910-42B5-B666-F8C2DA095755}">
   <dimension ref="A1:G115"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.28515625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="126.28515625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="69.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="1.28515625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="14.140625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="67.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="11.42578125" style="1"/>
+    <col min="1" max="1" width="76.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.26953125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="126.26953125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="69.7265625" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="1.26953125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="14.1796875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="67.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="11.453125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" customFormat="1" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="11" t="s">
         <v>195</v>
       </c>
@@ -7543,13 +7537,13 @@
       <c r="C1" s="14"/>
       <c r="D1" s="14"/>
     </row>
-    <row r="2" spans="1:7" customFormat="1" ht="21" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" customFormat="1" ht="21" x14ac:dyDescent="0.5">
       <c r="A2" s="11"/>
       <c r="B2" s="2"/>
       <c r="C2" s="14"/>
       <c r="D2" s="14"/>
     </row>
-    <row r="3" spans="1:7" s="36" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" s="36" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="34" t="s">
         <v>1</v>
       </c>
@@ -7567,7 +7561,7 @@
       </c>
       <c r="G3" s="1"/>
     </row>
-    <row r="4" spans="1:7" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="16" t="s">
         <v>115</v>
       </c>
@@ -7587,7 +7581,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="45" t="s">
         <v>105</v>
       </c>
@@ -7603,7 +7597,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="17" t="s">
         <v>116</v>
       </c>
@@ -7623,7 +7617,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="17" t="s">
         <v>117</v>
       </c>
@@ -7641,7 +7635,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="17" t="s">
         <v>119</v>
       </c>
@@ -7659,7 +7653,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="17" t="s">
         <v>118</v>
       </c>
@@ -7677,7 +7671,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="17" t="s">
         <v>120</v>
       </c>
@@ -7689,7 +7683,7 @@
       </c>
       <c r="D10" s="30"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="45" t="s">
         <v>8</v>
       </c>
@@ -7699,7 +7693,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="17" t="s">
         <v>121</v>
       </c>
@@ -7713,7 +7707,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="17" t="s">
         <v>122</v>
       </c>
@@ -7727,7 +7721,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="17" t="s">
         <v>123</v>
       </c>
@@ -7741,7 +7735,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="17" t="s">
         <v>124</v>
       </c>
@@ -7753,7 +7747,7 @@
       </c>
       <c r="D15" s="42"/>
     </row>
-    <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="17" t="s">
         <v>125</v>
       </c>
@@ -7767,7 +7761,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="17" t="s">
         <v>126</v>
       </c>
@@ -7781,7 +7775,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="45" t="s">
         <v>182</v>
       </c>
@@ -7791,7 +7785,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="17" t="s">
         <v>174</v>
       </c>
@@ -7803,7 +7797,7 @@
       </c>
       <c r="D19" s="30"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="17" t="s">
         <v>175</v>
       </c>
@@ -7815,7 +7809,7 @@
       </c>
       <c r="D20" s="30"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="17" t="s">
         <v>176</v>
       </c>
@@ -7827,7 +7821,7 @@
       </c>
       <c r="D21" s="30"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="17" t="s">
         <v>177</v>
       </c>
@@ -7839,7 +7833,7 @@
       </c>
       <c r="D22" s="30"/>
     </row>
-    <row r="23" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" s="17" t="s">
         <v>178</v>
       </c>
@@ -7853,7 +7847,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="17" t="s">
         <v>179</v>
       </c>
@@ -7865,7 +7859,7 @@
       </c>
       <c r="D24" s="30"/>
     </row>
-    <row r="25" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="17" t="s">
         <v>180</v>
       </c>
@@ -7877,7 +7871,7 @@
       </c>
       <c r="D25" s="30"/>
     </row>
-    <row r="26" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="18" t="s">
         <v>181</v>
       </c>
@@ -7889,7 +7883,7 @@
       </c>
       <c r="D26" s="38"/>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="41" t="s">
         <v>9</v>
       </c>
@@ -7897,7 +7891,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="17" t="s">
         <v>188</v>
       </c>
@@ -7911,7 +7905,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="17" t="s">
         <v>187</v>
       </c>
@@ -7923,7 +7917,7 @@
       </c>
       <c r="D29" s="30"/>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="17" t="s">
         <v>186</v>
       </c>
@@ -7937,7 +7931,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="17" t="s">
         <v>185</v>
       </c>
@@ -7949,7 +7943,7 @@
       </c>
       <c r="D31" s="30"/>
     </row>
-    <row r="32" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="A32" s="17" t="s">
         <v>184</v>
       </c>
@@ -7963,7 +7957,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A33" s="18" t="s">
         <v>183</v>
       </c>
@@ -7975,7 +7969,7 @@
       </c>
       <c r="D33" s="38"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="41" t="s">
         <v>3</v>
       </c>
@@ -7984,7 +7978,7 @@
       </c>
       <c r="E34" s="2"/>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="17" t="s">
         <v>189</v>
       </c>
@@ -7999,7 +7993,7 @@
       </c>
       <c r="E35" s="2"/>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="17" t="s">
         <v>190</v>
       </c>
@@ -8014,7 +8008,7 @@
       </c>
       <c r="E36" s="2"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="17" t="s">
         <v>191</v>
       </c>
@@ -8029,7 +8023,7 @@
       </c>
       <c r="E37" s="2"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="17" t="s">
         <v>192</v>
       </c>
@@ -8042,7 +8036,7 @@
       <c r="D38" s="30"/>
       <c r="E38" s="2"/>
     </row>
-    <row r="39" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A39" s="17" t="s">
         <v>193</v>
       </c>
@@ -8057,7 +8051,7 @@
       </c>
       <c r="E39" s="2"/>
     </row>
-    <row r="40" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A40" s="17" t="s">
         <v>194</v>
       </c>
@@ -8072,7 +8066,7 @@
       </c>
       <c r="E40" s="2"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="21" t="s">
         <v>14</v>
       </c>
@@ -8086,7 +8080,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="56" t="s">
         <v>12</v>
       </c>
@@ -8098,7 +8092,7 @@
       </c>
       <c r="D42" s="59"/>
     </row>
-    <row r="43" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A43" s="47" t="s">
         <v>6</v>
       </c>
@@ -8112,7 +8106,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="40" t="s">
         <v>106</v>
       </c>
@@ -8122,7 +8116,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="17" t="s">
         <v>127</v>
       </c>
@@ -8134,7 +8128,7 @@
       </c>
       <c r="D45" s="30"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="17" t="s">
         <v>128</v>
       </c>
@@ -8146,7 +8140,7 @@
       </c>
       <c r="D46" s="30"/>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="17" t="s">
         <v>129</v>
       </c>
@@ -8158,7 +8152,7 @@
       </c>
       <c r="D47" s="30"/>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="17" t="s">
         <v>130</v>
       </c>
@@ -8170,7 +8164,7 @@
       </c>
       <c r="D48" s="24"/>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" s="17" t="s">
         <v>131</v>
       </c>
@@ -8182,7 +8176,7 @@
       </c>
       <c r="D49" s="30"/>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" s="17" t="s">
         <v>132</v>
       </c>
@@ -8194,7 +8188,7 @@
       </c>
       <c r="D50" s="30"/>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" s="17" t="s">
         <v>133</v>
       </c>
@@ -8206,7 +8200,7 @@
       </c>
       <c r="D51" s="30"/>
     </row>
-    <row r="52" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="17" t="s">
         <v>134</v>
       </c>
@@ -8218,7 +8212,7 @@
       </c>
       <c r="D52" s="30"/>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" s="17" t="s">
         <v>135</v>
       </c>
@@ -8230,7 +8224,7 @@
       </c>
       <c r="D53" s="30"/>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" s="17" t="s">
         <v>136</v>
       </c>
@@ -8242,7 +8236,7 @@
       </c>
       <c r="D54" s="30"/>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" s="17" t="s">
         <v>137</v>
       </c>
@@ -8254,7 +8248,7 @@
       </c>
       <c r="D55" s="30"/>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" s="17" t="s">
         <v>138</v>
       </c>
@@ -8266,7 +8260,7 @@
       </c>
       <c r="D56" s="30"/>
     </row>
-    <row r="57" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="17" t="s">
         <v>139</v>
       </c>
@@ -8278,7 +8272,7 @@
       </c>
       <c r="D57" s="30"/>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" s="17" t="s">
         <v>140</v>
       </c>
@@ -8290,7 +8284,7 @@
       </c>
       <c r="D58" s="30"/>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" s="17" t="s">
         <v>141</v>
       </c>
@@ -8302,7 +8296,7 @@
       </c>
       <c r="D59" s="30"/>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" s="17" t="s">
         <v>142</v>
       </c>
@@ -8314,7 +8308,7 @@
       </c>
       <c r="D60" s="30"/>
     </row>
-    <row r="61" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" s="17" t="s">
         <v>143</v>
       </c>
@@ -8326,7 +8320,7 @@
       </c>
       <c r="D61" s="30"/>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" s="17" t="s">
         <v>144</v>
       </c>
@@ -8338,7 +8332,7 @@
       </c>
       <c r="D62" s="30"/>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" s="17" t="s">
         <v>145</v>
       </c>
@@ -8350,7 +8344,7 @@
       </c>
       <c r="D63" s="30"/>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" s="17" t="s">
         <v>146</v>
       </c>
@@ -8362,7 +8356,7 @@
       </c>
       <c r="D64" s="30"/>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" s="17" t="s">
         <v>147</v>
       </c>
@@ -8374,7 +8368,7 @@
       </c>
       <c r="D65" s="30"/>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" s="17" t="s">
         <v>148</v>
       </c>
@@ -8386,7 +8380,7 @@
       </c>
       <c r="D66" s="30"/>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" s="17" t="s">
         <v>149</v>
       </c>
@@ -8398,7 +8392,7 @@
       </c>
       <c r="D67" s="30"/>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A68" s="17" t="s">
         <v>150</v>
       </c>
@@ -8410,7 +8404,7 @@
       </c>
       <c r="D68" s="30"/>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A69" s="17" t="s">
         <v>151</v>
       </c>
@@ -8422,7 +8416,7 @@
       </c>
       <c r="D69" s="30"/>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A70" s="17" t="s">
         <v>152</v>
       </c>
@@ -8434,7 +8428,7 @@
       </c>
       <c r="D70" s="30"/>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A71" s="17" t="s">
         <v>153</v>
       </c>
@@ -8446,7 +8440,7 @@
       </c>
       <c r="D71" s="30"/>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A72" s="17" t="s">
         <v>154</v>
       </c>
@@ -8458,7 +8452,7 @@
       </c>
       <c r="D72" s="30"/>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A73" s="17" t="s">
         <v>155</v>
       </c>
@@ -8470,7 +8464,7 @@
       </c>
       <c r="D73" s="30"/>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A74" s="17" t="s">
         <v>156</v>
       </c>
@@ -8482,7 +8476,7 @@
       </c>
       <c r="D74" s="30"/>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A75" s="17" t="s">
         <v>157</v>
       </c>
@@ -8494,7 +8488,7 @@
       </c>
       <c r="D75" s="30"/>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76" s="17" t="s">
         <v>158</v>
       </c>
@@ -8506,7 +8500,7 @@
       </c>
       <c r="D76" s="30"/>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77" s="39" t="s">
         <v>159</v>
       </c>
@@ -8518,7 +8512,7 @@
       </c>
       <c r="D77" s="30"/>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A78" s="39" t="s">
         <v>160</v>
       </c>
@@ -8530,7 +8524,7 @@
       </c>
       <c r="D78" s="30"/>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A79" s="17" t="s">
         <v>161</v>
       </c>
@@ -8542,7 +8536,7 @@
       </c>
       <c r="D79" s="30"/>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80" s="17" t="s">
         <v>162</v>
       </c>
@@ -8554,7 +8548,7 @@
       </c>
       <c r="D80" s="30"/>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="17" t="s">
         <v>163</v>
       </c>
@@ -8566,7 +8560,7 @@
       </c>
       <c r="D81" s="30"/>
     </row>
-    <row r="82" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A82" s="17" t="s">
         <v>164</v>
       </c>
@@ -8578,7 +8572,7 @@
       </c>
       <c r="D82" s="30"/>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" s="17" t="s">
         <v>165</v>
       </c>
@@ -8590,7 +8584,7 @@
       </c>
       <c r="D83" s="30"/>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" s="17" t="s">
         <v>166</v>
       </c>
@@ -8602,7 +8596,7 @@
       </c>
       <c r="D84" s="30"/>
     </row>
-    <row r="85" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A85" s="17" t="s">
         <v>167</v>
       </c>
@@ -8616,7 +8610,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="86" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A86" s="17" t="s">
         <v>168</v>
       </c>
@@ -8630,7 +8624,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="53" t="s">
         <v>171</v>
       </c>
@@ -8642,7 +8636,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="88" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:5" ht="73" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A88" s="39" t="s">
         <v>169</v>
       </c>
@@ -8656,7 +8650,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="89" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:5" ht="73" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A89" s="22" t="s">
         <v>170</v>
       </c>
@@ -8670,13 +8664,13 @@
         <v>204</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" s="25"/>
       <c r="B91" s="29"/>
       <c r="C91" s="29"/>
       <c r="D91" s="29"/>
     </row>
-    <row r="93" spans="1:5" customFormat="1" ht="21" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5" customFormat="1" ht="21" x14ac:dyDescent="0.35">
       <c r="A93" s="64" t="s">
         <v>56</v>
       </c>
@@ -8684,7 +8678,7 @@
       <c r="C93" s="10"/>
       <c r="D93" s="10"/>
     </row>
-    <row r="94" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A94" s="3" t="s">
         <v>1</v>
       </c>
@@ -8698,7 +8692,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95" s="46" t="s">
         <v>21</v>
       </c>
@@ -8712,7 +8706,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="96" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A96" s="17" t="s">
         <v>10</v>
       </c>
@@ -8727,7 +8721,7 @@
       </c>
       <c r="E96" s="2"/>
     </row>
-    <row r="97" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A97" s="47" t="s">
         <v>6</v>
       </c>
@@ -8741,7 +8735,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="98" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A98" s="39" t="s">
         <v>103</v>
       </c>
@@ -8756,7 +8750,7 @@
       </c>
       <c r="E98" s="4"/>
     </row>
-    <row r="99" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:5" ht="73" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A99" s="22" t="s">
         <v>104</v>
       </c>
@@ -8771,7 +8765,7 @@
       </c>
       <c r="E99" s="4"/>
     </row>
-    <row r="115" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A115" s="1"/>
       <c r="C115" s="4"/>
       <c r="E115" s="1"/>
@@ -8784,6 +8778,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101008B2C02A454474E49AF1E88C4BB44217A" ma:contentTypeVersion="2" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="9e15e66e190a04cb6a1b159509d80e16">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="75c7dcee-517e-489f-adec-4c479389f6c8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="41966a1257569f694d2354f349558ce6" ns2:_="">
     <xsd:import namespace="75c7dcee-517e-489f-adec-4c479389f6c8"/>
@@ -8931,35 +8940,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0F56C80-3573-454E-96BA-4B4F570D915F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5890D2DC-C0F6-4046-AE53-B2F6CA431A90}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="75c7dcee-517e-489f-adec-4c479389f6c8"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -8981,9 +8965,19 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5890D2DC-C0F6-4046-AE53-B2F6CA431A90}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0F56C80-3573-454E-96BA-4B4F570D915F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="75c7dcee-517e-489f-adec-4c479389f6c8"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>